<commit_message>
import and start cleaning; fixed typos in XLSX
</commit_message>
<xml_diff>
--- a/data/AURecruit.xlsx
+++ b/data/AURecruit.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/djo/Dropbox/Personal/Studies/0-Grad School/MEM Program/!Research/Diss/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/djo/dev/au/au_diss/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AF746AE-B461-1343-8F77-8AB218EB9B32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F70EE2A-84F3-C247-A7C3-FF99DAD6506B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="23040" windowHeight="25420" xr2:uid="{9D3AC3E5-42CD-5B4C-9A6D-E91B574DC308}"/>
   </bookViews>
@@ -53,9 +53,6 @@
     <t>Ethnicity</t>
   </si>
   <si>
-    <t>Coutnry</t>
-  </si>
-  <si>
     <t>Language</t>
   </si>
   <si>
@@ -209,9 +206,6 @@
     <t>H</t>
   </si>
   <si>
-    <t>Austrailia</t>
-  </si>
-  <si>
     <t>PYERGO</t>
   </si>
   <si>
@@ -249,6 +243,12 @@
   </si>
   <si>
     <t>ME</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>Australia</t>
   </si>
 </sst>
 </file>
@@ -292,12 +292,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -628,69 +625,69 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="19" width="10.83203125" style="1"/>
-    <col min="20" max="20" width="53.1640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="53.1640625" style="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="4" t="s">
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="4" t="s">
+      <c r="F1" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="M1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="O1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="P1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="Q1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="R1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="S1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="5" t="s">
-        <v>63</v>
+      <c r="T1" s="4" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.2">
@@ -698,7 +695,7 @@
         <v>1001</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C2" s="1">
         <v>20</v>
@@ -710,19 +707,19 @@
         <v>2</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H2" s="1">
         <v>3</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K2" s="1">
         <v>2</v>
@@ -731,25 +728,25 @@
         <v>1</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q2" s="1">
         <v>68</v>
       </c>
       <c r="R2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="S2" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.2">
@@ -757,7 +754,7 @@
         <v>1003</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" s="1">
         <v>21</v>
@@ -769,20 +766,20 @@
         <v>2</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H3" s="1">
         <v>3</v>
       </c>
       <c r="I3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J3" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="K3" s="1">
         <v>2</v>
       </c>
@@ -790,25 +787,25 @@
         <v>1</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R3" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="S3" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.2">
@@ -816,31 +813,31 @@
         <v>1005</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="1">
+        <v>28</v>
+      </c>
+      <c r="D4" s="1">
+        <v>2</v>
+      </c>
+      <c r="E4" s="1">
+        <v>2</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C4" s="1">
-        <v>28</v>
-      </c>
-      <c r="D4" s="1">
-        <v>2</v>
-      </c>
-      <c r="E4" s="1">
-        <v>2</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="G4" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H4" s="1">
         <v>6</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K4" s="1">
         <v>1</v>
@@ -849,25 +846,25 @@
         <v>1</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R4" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="S4" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.2">
@@ -875,7 +872,7 @@
         <v>1006</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C5" s="1">
         <v>32</v>
@@ -887,19 +884,19 @@
         <v>2</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H5" s="1">
         <v>7</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K5" s="1">
         <v>1</v>
@@ -908,25 +905,25 @@
         <v>1</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="S5" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.2">
@@ -934,7 +931,7 @@
         <v>1007</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C6" s="1">
         <v>45</v>
@@ -946,20 +943,20 @@
         <v>2</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H6" s="1">
         <v>5</v>
       </c>
       <c r="I6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J6" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="J6" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="K6" s="1">
         <v>2</v>
       </c>
@@ -967,25 +964,25 @@
         <v>1</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="S6" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.2">
@@ -993,7 +990,7 @@
         <v>1008</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C7" s="1">
         <v>19</v>
@@ -1005,19 +1002,19 @@
         <v>2</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H7" s="1">
         <v>3</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K7" s="1">
         <v>2</v>
@@ -1026,25 +1023,25 @@
         <v>1</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R7" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="S7" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.2">
@@ -1052,7 +1049,7 @@
         <v>1009</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8" s="1">
         <v>21</v>
@@ -1064,19 +1061,19 @@
         <v>1</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H8" s="1">
         <v>3</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K8" s="1">
         <v>2</v>
@@ -1085,25 +1082,25 @@
         <v>1</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.2">
@@ -1111,7 +1108,7 @@
         <v>1010</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C9" s="1">
         <v>23</v>
@@ -1123,19 +1120,19 @@
         <v>2</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H9" s="1">
         <v>3</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K9" s="1">
         <v>1</v>
@@ -1144,25 +1141,25 @@
         <v>3</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.2">
@@ -1170,10 +1167,10 @@
         <v>1011</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D10" s="1">
         <v>5</v>
@@ -1182,19 +1179,19 @@
         <v>2</v>
       </c>
       <c r="F10" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G10" s="1" t="s">
-        <v>37</v>
-      </c>
       <c r="H10" s="1">
         <v>3</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K10" s="1">
         <v>1</v>
@@ -1203,25 +1200,25 @@
         <v>1</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R10" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="S10" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.2">
@@ -1229,7 +1226,7 @@
         <v>1012</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C11" s="1">
         <v>42</v>
@@ -1241,46 +1238,46 @@
         <v>2</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H11" s="1">
         <v>6</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K11" s="1">
+        <v>2</v>
+      </c>
+      <c r="L11" s="1">
+        <v>1</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="P11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="R11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="S11" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="K11" s="1">
-        <v>2</v>
-      </c>
-      <c r="L11" s="1">
-        <v>1</v>
-      </c>
-      <c r="M11" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="N11" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="O11" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="P11" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q11" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="R11" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="S11" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.2">
@@ -1288,7 +1285,7 @@
         <v>1013</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C12" s="1">
         <v>21</v>
@@ -1300,19 +1297,19 @@
         <v>2</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H12" s="1">
         <v>3</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K12" s="1">
         <v>4</v>
@@ -1321,25 +1318,25 @@
         <v>3</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="S12" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.2">
@@ -1347,7 +1344,7 @@
         <v>1014</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C13" s="1">
         <v>19</v>
@@ -1359,19 +1356,19 @@
         <v>2</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H13" s="1">
         <v>3</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K13" s="1">
         <v>2</v>
@@ -1380,25 +1377,25 @@
         <v>1</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q13" s="1">
         <v>66</v>
       </c>
       <c r="R13" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="S13" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.2">
@@ -1406,7 +1403,7 @@
         <v>1015</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C14" s="1">
         <v>20</v>
@@ -1418,19 +1415,19 @@
         <v>2</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H14" s="1">
         <v>3</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K14" s="1">
         <v>3</v>
@@ -1439,25 +1436,25 @@
         <v>1</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q14" s="1">
         <v>66</v>
       </c>
       <c r="R14" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="S14" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.2">
@@ -1465,7 +1462,7 @@
         <v>1016</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C15" s="1">
         <v>22</v>
@@ -1477,19 +1474,19 @@
         <v>2</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H15" s="1">
         <v>4</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K15" s="1">
         <v>2</v>
@@ -1498,25 +1495,25 @@
         <v>4</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q15" s="1">
         <v>74</v>
       </c>
       <c r="R15" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="S15" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.2">
@@ -1524,7 +1521,7 @@
         <v>1017</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C16" s="1">
         <v>24</v>
@@ -1536,19 +1533,19 @@
         <v>2</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H16" s="1">
         <v>6</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K16" s="1">
         <v>3</v>
@@ -1557,25 +1554,25 @@
         <v>2</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R16" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="S16" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.2">
@@ -1583,7 +1580,7 @@
         <v>1018</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C17" s="1">
         <v>20</v>
@@ -1595,20 +1592,20 @@
         <v>2</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H17" s="1">
         <v>3</v>
       </c>
       <c r="I17" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="J17" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J17" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="K17" s="1">
         <v>3</v>
       </c>
@@ -1616,25 +1613,25 @@
         <v>1</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q17" s="1">
         <v>71</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.2">
@@ -1642,7 +1639,7 @@
         <v>1019</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C18" s="1">
         <v>21</v>
@@ -1654,19 +1651,19 @@
         <v>2</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H18" s="1">
         <v>3</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K18" s="1">
         <v>3</v>
@@ -1675,25 +1672,25 @@
         <v>2</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q18" s="1">
         <v>65</v>
       </c>
       <c r="R18" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S18" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.2">
@@ -1701,7 +1698,7 @@
         <v>1020</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C19" s="1">
         <v>20</v>
@@ -1713,19 +1710,19 @@
         <v>2</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H19" s="1">
         <v>3</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="K19" s="1">
         <v>2</v>
@@ -1734,25 +1731,25 @@
         <v>1</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q19" s="1">
         <v>70</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S19" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.2">
@@ -1760,10 +1757,10 @@
         <v>1021</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D20" s="1">
         <v>5</v>
@@ -1772,19 +1769,19 @@
         <v>2</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H20" s="1">
         <v>3</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="K20" s="1">
         <v>2</v>
@@ -1793,16 +1790,16 @@
         <v>1</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P20" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q20" s="1">
         <v>71</v>
@@ -1811,7 +1808,7 @@
         <v>5</v>
       </c>
       <c r="S20" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.2">
@@ -1819,7 +1816,7 @@
         <v>1022</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C21" s="1">
         <v>21</v>
@@ -1831,19 +1828,19 @@
         <v>2</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H21" s="1">
         <v>3</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K21" s="1">
         <v>3</v>
@@ -1852,16 +1849,16 @@
         <v>4</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q21" s="1">
         <v>76</v>
@@ -1870,7 +1867,7 @@
         <v>5</v>
       </c>
       <c r="S21" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.2">
@@ -1878,7 +1875,7 @@
         <v>1023</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C22" s="1">
         <v>21</v>
@@ -1890,19 +1887,19 @@
         <v>2</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H22" s="1">
         <v>3</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K22" s="1">
         <v>1</v>
@@ -1911,16 +1908,16 @@
         <v>1</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O22" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P22" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q22" s="1">
         <v>68</v>
@@ -1929,7 +1926,7 @@
         <v>5</v>
       </c>
       <c r="S22" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.2">
@@ -1937,7 +1934,7 @@
         <v>1024</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C23" s="1">
         <v>20</v>
@@ -1946,22 +1943,22 @@
         <v>5</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H23" s="1">
         <v>3</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K23" s="1">
         <v>2</v>
@@ -1970,16 +1967,16 @@
         <v>1</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O23" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P23" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q23" s="1">
         <v>73</v>
@@ -1988,7 +1985,7 @@
         <v>5</v>
       </c>
       <c r="S23" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.2">
@@ -1996,7 +1993,7 @@
         <v>1025</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C24" s="1">
         <v>19</v>
@@ -2008,19 +2005,19 @@
         <v>2</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H24" s="1">
         <v>3</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K24" s="1">
         <v>1</v>
@@ -2029,25 +2026,25 @@
         <v>2</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N24" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="O24" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P24" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q24" s="1">
         <v>64</v>
       </c>
       <c r="R24" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S24" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.2">
@@ -2055,7 +2052,7 @@
         <v>1026</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C25" s="1">
         <v>20</v>
@@ -2067,46 +2064,46 @@
         <v>2</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H25" s="1">
         <v>3</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J25" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K25" s="1">
+        <v>1</v>
+      </c>
+      <c r="L25" s="1">
+        <v>1</v>
+      </c>
+      <c r="M25" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="N25" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K25" s="1">
-        <v>1</v>
-      </c>
-      <c r="L25" s="1">
-        <v>1</v>
-      </c>
-      <c r="M25" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="N25" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="O25" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P25" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q25" s="1">
         <v>67</v>
       </c>
       <c r="R25" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="S25" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.2">
@@ -2114,7 +2111,7 @@
         <v>1027</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C26" s="1">
         <v>20</v>
@@ -2126,19 +2123,19 @@
         <v>2</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H26" s="1">
         <v>3</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K26" s="1">
         <v>1</v>
@@ -2147,16 +2144,16 @@
         <v>3</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O26" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P26" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q26" s="1">
         <v>67</v>
@@ -2165,7 +2162,7 @@
         <v>5</v>
       </c>
       <c r="S26" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.2">
@@ -2173,7 +2170,7 @@
         <v>1028</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C27" s="1">
         <v>20</v>
@@ -2185,19 +2182,19 @@
         <v>2</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H27" s="1">
         <v>3</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K27" s="1">
         <v>1</v>
@@ -2206,25 +2203,25 @@
         <v>1</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O27" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P27" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q27" s="1">
         <v>66</v>
       </c>
       <c r="R27" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S27" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.2">
@@ -2232,7 +2229,7 @@
         <v>1029</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C28" s="1">
         <v>22</v>
@@ -2244,19 +2241,19 @@
         <v>2</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H28" s="1">
         <v>3</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K28" s="1">
         <v>2</v>
@@ -2265,25 +2262,25 @@
         <v>1</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="O28" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P28" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q28" s="1">
         <v>68</v>
       </c>
       <c r="R28" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S28" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.2">
@@ -2291,7 +2288,7 @@
         <v>1030</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C29" s="1">
         <v>21</v>
@@ -2303,19 +2300,19 @@
         <v>2</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H29" s="1">
         <v>3</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K29" s="1">
         <v>1</v>
@@ -2324,16 +2321,16 @@
         <v>2</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O29" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P29" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q29" s="1">
         <v>63</v>
@@ -2342,7 +2339,7 @@
         <v>5</v>
       </c>
       <c r="S29" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.2">
@@ -2350,7 +2347,7 @@
         <v>1031</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C30" s="1">
         <v>19</v>
@@ -2362,19 +2359,19 @@
         <v>1</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H30" s="1">
         <v>3</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K30" s="1">
         <v>3</v>
@@ -2383,25 +2380,25 @@
         <v>1</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="O30" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P30" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q30" s="1">
         <v>71</v>
       </c>
       <c r="R30" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S30" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.2">
@@ -2409,7 +2406,7 @@
         <v>1032</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C31" s="1">
         <v>19</v>
@@ -2421,19 +2418,19 @@
         <v>2</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H31" s="1">
         <v>3</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K31" s="1">
         <v>2</v>
@@ -2442,16 +2439,16 @@
         <v>1</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="O31" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P31" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q31" s="1">
         <v>66</v>
@@ -2460,7 +2457,7 @@
         <v>5</v>
       </c>
       <c r="S31" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.2">
@@ -2468,7 +2465,7 @@
         <v>1033</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C32" s="1">
         <v>21</v>
@@ -2480,19 +2477,19 @@
         <v>2</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H32" s="1">
         <v>3</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="K32" s="1">
         <v>2</v>
@@ -2501,25 +2498,25 @@
         <v>1</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O32" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P32" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q32" s="1">
         <v>69</v>
       </c>
       <c r="R32" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S32" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.2">
@@ -2527,7 +2524,7 @@
         <v>1034</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C33" s="1">
         <v>20</v>
@@ -2539,19 +2536,19 @@
         <v>2</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H33" s="1">
         <v>3</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K33" s="1">
         <v>1</v>
@@ -2560,16 +2557,16 @@
         <v>1</v>
       </c>
       <c r="M33" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O33" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P33" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q33" s="1">
         <v>65</v>
@@ -2578,7 +2575,7 @@
         <v>5</v>
       </c>
       <c r="S33" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.2">
@@ -2586,7 +2583,7 @@
         <v>1035</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C34" s="1">
         <v>21</v>
@@ -2598,19 +2595,19 @@
         <v>2</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H34" s="1">
         <v>3</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K34" s="1">
         <v>2</v>
@@ -2619,16 +2616,16 @@
         <v>2</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O34" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P34" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q34" s="1">
         <v>68</v>
@@ -2637,7 +2634,7 @@
         <v>5</v>
       </c>
       <c r="S34" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.2">
@@ -2645,7 +2642,7 @@
         <v>1036</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C35" s="1">
         <v>21</v>
@@ -2657,19 +2654,19 @@
         <v>2</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H35" s="1">
         <v>3</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K35" s="1">
         <v>1</v>
@@ -2678,25 +2675,25 @@
         <v>2</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O35" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P35" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q35" s="1">
         <v>62</v>
       </c>
       <c r="R35" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S35" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.2">
@@ -2704,7 +2701,7 @@
         <v>1037</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C36" s="1">
         <v>43</v>
@@ -2716,19 +2713,19 @@
         <v>2</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H36" s="1">
         <v>6</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K36" s="1">
         <v>1</v>
@@ -2737,25 +2734,25 @@
         <v>4</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O36" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P36" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q36" s="1">
         <v>70</v>
       </c>
       <c r="R36" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="S36" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.2">
@@ -2763,7 +2760,7 @@
         <v>1038</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C37" s="1">
         <v>20</v>
@@ -2775,19 +2772,19 @@
         <v>2</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H37" s="1">
         <v>3</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K37" s="1">
         <v>2</v>
@@ -2796,16 +2793,16 @@
         <v>1</v>
       </c>
       <c r="M37" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O37" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P37" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q37" s="1">
         <v>63</v>
@@ -2814,7 +2811,7 @@
         <v>5</v>
       </c>
       <c r="S37" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.2">
@@ -2822,7 +2819,7 @@
         <v>1039</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C38" s="1">
         <v>20</v>
@@ -2834,19 +2831,19 @@
         <v>2</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H38" s="1">
         <v>3</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K38" s="1">
         <v>2</v>
@@ -2855,16 +2852,16 @@
         <v>1</v>
       </c>
       <c r="M38" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N38" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O38" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P38" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q38" s="1">
         <v>64</v>
@@ -2873,7 +2870,7 @@
         <v>5</v>
       </c>
       <c r="S38" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.2">
@@ -2881,7 +2878,7 @@
         <v>1040</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C39" s="1">
         <v>21</v>
@@ -2893,19 +2890,19 @@
         <v>2</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H39" s="1">
         <v>3</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K39" s="1">
         <v>2</v>
@@ -2914,16 +2911,16 @@
         <v>2</v>
       </c>
       <c r="M39" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N39" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O39" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P39" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q39" s="1">
         <v>72</v>
@@ -2932,7 +2929,7 @@
         <v>10</v>
       </c>
       <c r="S39" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.2">
@@ -2940,7 +2937,7 @@
         <v>1041</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C40" s="1">
         <v>20</v>
@@ -2952,19 +2949,19 @@
         <v>2</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H40" s="1">
         <v>3</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K40" s="1">
         <v>2</v>
@@ -2973,16 +2970,16 @@
         <v>2</v>
       </c>
       <c r="M40" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N40" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O40" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P40" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q40" s="1">
         <v>66</v>
@@ -2991,7 +2988,7 @@
         <v>10</v>
       </c>
       <c r="S40" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.2">
@@ -2999,7 +2996,7 @@
         <v>1042</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C41" s="1">
         <v>20</v>
@@ -3011,19 +3008,19 @@
         <v>2</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H41" s="1">
         <v>3</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K41" s="1">
         <v>3</v>
@@ -3032,16 +3029,16 @@
         <v>1</v>
       </c>
       <c r="M41" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N41" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O41" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P41" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q41" s="1">
         <v>75</v>
@@ -3050,7 +3047,7 @@
         <v>5</v>
       </c>
       <c r="S41" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.2">
@@ -3058,7 +3055,7 @@
         <v>1043</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C42" s="1">
         <v>20</v>
@@ -3070,19 +3067,19 @@
         <v>2</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H42" s="1">
         <v>3</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K42" s="1">
         <v>2</v>
@@ -3091,25 +3088,25 @@
         <v>1</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O42" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P42" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q42" s="1">
         <v>74</v>
       </c>
       <c r="R42" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S42" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.2">
@@ -3117,7 +3114,7 @@
         <v>1044</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C43" s="1">
         <v>19</v>
@@ -3129,19 +3126,19 @@
         <v>2</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H43" s="1">
         <v>3</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K43" s="1">
         <v>1</v>
@@ -3150,25 +3147,25 @@
         <v>1</v>
       </c>
       <c r="M43" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N43" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O43" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P43" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q43" s="1">
         <v>62</v>
       </c>
       <c r="R43" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S43" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.2">
@@ -3176,7 +3173,7 @@
         <v>1045</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C44" s="1">
         <v>21</v>
@@ -3188,19 +3185,19 @@
         <v>2</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H44" s="1">
         <v>3</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K44" s="1">
         <v>1</v>
@@ -3209,25 +3206,25 @@
         <v>3</v>
       </c>
       <c r="M44" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N44" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O44" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P44" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q44" s="1">
         <v>69</v>
       </c>
       <c r="R44" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="S44" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.2">
@@ -3235,7 +3232,7 @@
         <v>1046</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C45" s="1">
         <v>19</v>
@@ -3247,19 +3244,19 @@
         <v>2</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H45" s="1">
         <v>3</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K45" s="1">
         <v>2</v>
@@ -3268,25 +3265,25 @@
         <v>1</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N45" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O45" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P45" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q45" s="1">
         <v>75</v>
       </c>
       <c r="R45" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S45" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.2">
@@ -3294,7 +3291,7 @@
         <v>1047</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C46" s="1">
         <v>20</v>
@@ -3306,19 +3303,19 @@
         <v>2</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H46" s="1">
         <v>3</v>
       </c>
       <c r="I46" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K46" s="1">
         <v>2</v>
@@ -3327,16 +3324,16 @@
         <v>3</v>
       </c>
       <c r="M46" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N46" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O46" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P46" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q46" s="1">
         <v>75</v>
@@ -3345,7 +3342,7 @@
         <v>5</v>
       </c>
       <c r="S46" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.2">
@@ -3353,7 +3350,7 @@
         <v>1048</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C47" s="1">
         <v>21</v>
@@ -3365,19 +3362,19 @@
         <v>2</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H47" s="1">
         <v>3</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K47" s="1">
         <v>4</v>
@@ -3386,16 +3383,16 @@
         <v>1</v>
       </c>
       <c r="M47" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N47" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O47" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P47" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q47" s="1">
         <v>72</v>
@@ -3404,7 +3401,7 @@
         <v>10</v>
       </c>
       <c r="S47" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.2">
@@ -3412,7 +3409,7 @@
         <v>1049</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C48" s="1">
         <v>20</v>
@@ -3424,19 +3421,19 @@
         <v>2</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H48" s="1">
         <v>3</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J48" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K48" s="1">
         <v>4</v>
@@ -3445,16 +3442,16 @@
         <v>1</v>
       </c>
       <c r="M48" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N48" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O48" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P48" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q48" s="1">
         <v>72</v>
@@ -3463,7 +3460,7 @@
         <v>5</v>
       </c>
       <c r="S48" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="49" spans="1:20" x14ac:dyDescent="0.2">
@@ -3471,7 +3468,7 @@
         <v>1050</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C49" s="1">
         <v>19</v>
@@ -3483,19 +3480,19 @@
         <v>2</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H49" s="1">
         <v>4</v>
       </c>
       <c r="I49" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J49" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K49" s="1">
         <v>3</v>
@@ -3504,25 +3501,25 @@
         <v>2</v>
       </c>
       <c r="M49" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N49" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O49" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P49" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q49" s="1">
         <v>71</v>
       </c>
       <c r="R49" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S49" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="50" spans="1:20" x14ac:dyDescent="0.2">
@@ -3530,7 +3527,7 @@
         <v>1051</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C50" s="1">
         <v>19</v>
@@ -3542,19 +3539,19 @@
         <v>2</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H50" s="1">
         <v>3</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J50" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K50" s="1">
         <v>1</v>
@@ -3563,16 +3560,16 @@
         <v>1</v>
       </c>
       <c r="M50" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N50" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O50" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P50" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q50" s="1">
         <v>62</v>
@@ -3581,7 +3578,7 @@
         <v>5</v>
       </c>
       <c r="S50" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="51" spans="1:20" x14ac:dyDescent="0.2">
@@ -3589,7 +3586,7 @@
         <v>1052</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C51" s="1">
         <v>20</v>
@@ -3601,19 +3598,19 @@
         <v>2</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H51" s="1">
         <v>3</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K51" s="1">
         <v>1</v>
@@ -3622,25 +3619,25 @@
         <v>1</v>
       </c>
       <c r="M51" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N51" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O51" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P51" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q51" s="1">
         <v>74</v>
       </c>
       <c r="R51" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="S51" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="52" spans="1:20" x14ac:dyDescent="0.2">
@@ -3648,7 +3645,7 @@
         <v>1053</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C52" s="1">
         <v>47</v>
@@ -3660,19 +3657,19 @@
         <v>2</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H52" s="1">
         <v>7</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K52" s="1">
         <v>2</v>
@@ -3681,25 +3678,25 @@
         <v>1</v>
       </c>
       <c r="M52" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N52" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="O52" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P52" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q52" s="1">
         <v>64</v>
       </c>
       <c r="R52" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S52" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="53" spans="1:20" x14ac:dyDescent="0.2">
@@ -3707,7 +3704,7 @@
         <v>1054</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C53" s="1">
         <v>21</v>
@@ -3719,19 +3716,19 @@
         <v>2</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H53" s="1">
         <v>3</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K53" s="1">
         <v>2</v>
@@ -3740,25 +3737,25 @@
         <v>1</v>
       </c>
       <c r="M53" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N53" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O53" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P53" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q53" s="1">
         <v>69</v>
       </c>
       <c r="R53" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S53" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="54" spans="1:20" x14ac:dyDescent="0.2">
@@ -3766,7 +3763,7 @@
         <v>1055</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C54" s="1">
         <v>19</v>
@@ -3778,19 +3775,19 @@
         <v>2</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H54" s="1">
         <v>3</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K54" s="1">
         <v>2</v>
@@ -3799,25 +3796,25 @@
         <v>1</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N54" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O54" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P54" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q54" s="1">
         <v>72</v>
       </c>
       <c r="R54" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S54" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="55" spans="1:20" x14ac:dyDescent="0.2">
@@ -3825,7 +3822,7 @@
         <v>1056</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C55" s="1">
         <v>20</v>
@@ -3837,46 +3834,46 @@
         <v>2</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H55" s="1">
         <v>3</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K55" s="1">
         <v>1</v>
       </c>
-      <c r="L55" s="2">
+      <c r="L55" s="1">
         <v>4</v>
       </c>
       <c r="M55" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N55" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O55" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P55" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q55" s="1">
         <v>64</v>
       </c>
       <c r="R55" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S55" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="56" spans="1:20" x14ac:dyDescent="0.2">
@@ -3884,7 +3881,7 @@
         <v>1057</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C56" s="1">
         <v>20</v>
@@ -3896,19 +3893,19 @@
         <v>2</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H56" s="1">
         <v>3</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K56" s="1">
         <v>1</v>
@@ -3917,25 +3914,25 @@
         <v>3</v>
       </c>
       <c r="M56" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N56" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O56" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P56" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q56" s="1">
         <v>64</v>
       </c>
       <c r="R56" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S56" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="57" spans="1:20" x14ac:dyDescent="0.2">
@@ -3943,7 +3940,7 @@
         <v>1058</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C57" s="1">
         <v>33</v>
@@ -3955,46 +3952,46 @@
         <v>2</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H57" s="1">
         <v>7</v>
       </c>
       <c r="I57" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="J57" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K57" s="1">
+        <v>1</v>
+      </c>
+      <c r="L57" s="1">
+        <v>1</v>
+      </c>
+      <c r="M57" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="N57" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J57" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K57" s="1">
-        <v>1</v>
-      </c>
-      <c r="L57" s="1">
-        <v>1</v>
-      </c>
-      <c r="M57" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="N57" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="O57" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P57" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q57" s="1">
         <v>65</v>
       </c>
       <c r="R57" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S57" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="58" spans="1:20" x14ac:dyDescent="0.2">
@@ -4002,7 +3999,7 @@
         <v>1059</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C58" s="1">
         <v>21</v>
@@ -4014,19 +4011,19 @@
         <v>2</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H58" s="1">
         <v>3</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="K58" s="1">
         <v>4</v>
@@ -4035,25 +4032,25 @@
         <v>1</v>
       </c>
       <c r="M58" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N58" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O58" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P58" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q58" s="1">
         <v>74</v>
       </c>
       <c r="R58" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S58" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="59" spans="1:20" x14ac:dyDescent="0.2">
@@ -4061,7 +4058,7 @@
         <v>1060</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C59" s="1">
         <v>20</v>
@@ -4073,19 +4070,19 @@
         <v>2</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H59" s="1">
         <v>3</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J59" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K59" s="1">
         <v>1</v>
@@ -4094,16 +4091,16 @@
         <v>1</v>
       </c>
       <c r="M59" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N59" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O59" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P59" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="Q59" s="1">
         <v>64</v>
@@ -4112,10 +4109,10 @@
         <v>5</v>
       </c>
       <c r="S59" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="T59" s="6" t="s">
-        <v>64</v>
+        <v>56</v>
+      </c>
+      <c r="T59" s="5" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="60" spans="1:20" x14ac:dyDescent="0.2">
@@ -4123,7 +4120,7 @@
         <v>1061</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C60" s="1">
         <v>20</v>
@@ -4135,19 +4132,19 @@
         <v>2</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H60" s="1">
         <v>3</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J60" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K60" s="1">
         <v>2</v>
@@ -4156,25 +4153,25 @@
         <v>2</v>
       </c>
       <c r="M60" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N60" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O60" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P60" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q60" s="1">
         <v>66</v>
       </c>
       <c r="R60" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="S60" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="61" spans="1:20" x14ac:dyDescent="0.2">
@@ -4182,7 +4179,7 @@
         <v>1062</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C61" s="1">
         <v>40</v>
@@ -4194,19 +4191,19 @@
         <v>2</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H61" s="1">
         <v>6</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J61" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K61" s="1">
         <v>3</v>
@@ -4215,25 +4212,25 @@
         <v>1</v>
       </c>
       <c r="M61" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N61" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O61" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P61" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q61" s="1">
         <v>64</v>
       </c>
       <c r="R61" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S61" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="62" spans="1:20" x14ac:dyDescent="0.2">
@@ -4241,7 +4238,7 @@
         <v>1063</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C62" s="1">
         <v>32</v>
@@ -4253,19 +4250,19 @@
         <v>2</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H62" s="1">
         <v>6</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K62" s="1">
         <v>2</v>
@@ -4274,25 +4271,25 @@
         <v>1</v>
       </c>
       <c r="M62" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N62" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O62" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P62" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q62" s="1">
         <v>73</v>
       </c>
       <c r="R62" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="S62" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="63" spans="1:20" x14ac:dyDescent="0.2">
@@ -4300,7 +4297,7 @@
         <v>1064</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C63" s="1">
         <v>24</v>
@@ -4312,19 +4309,19 @@
         <v>2</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H63" s="1">
         <v>5</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="K63" s="1">
         <v>3</v>
@@ -4333,25 +4330,25 @@
         <v>3</v>
       </c>
       <c r="M63" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N63" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O63" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P63" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q63" s="1">
         <v>74</v>
       </c>
       <c r="R63" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="S63" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>